<commit_message>
Remove local-path metadata from source workbook
</commit_message>
<xml_diff>
--- a/data/reference/Utah_Construction_Data.xlsx
+++ b/data/reference/Utah_Construction_Data.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liqui\Documents\Codex\2026-10-01\referenced-chatgpt-conversation-this-is-an\outputs\utah-construction-data\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="11_D44F93DC579A51893B86095DFB5BC8FBED35EBDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>